<commit_message>
C3 2AFC uses deployed dual FUDGE (4,2) vs no_guidance (100 distinct pairs)
- switched C3 from isolated positive_only (59 pairs, 41% identical) to the
  full dual operating point (100 pairs, 0% identical) - tests the actual method
- analyze_c3 keys renamed prefer_positive -> prefer_dual
- refreshed rater_annotation_R1/R2/R3.xlsx

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/human_labeling/rater_annotation_R1.xlsx
+++ b/results/human_labeling/rater_annotation_R1.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -514,8 +514,16 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
+        <is>
+          <t>Sheet 'C3_pairwise_engagement': read the source and the two rewrites A and B; in the 'choice' cell pick the ONE you would be more likely to click (A or B).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Sheet 'C3_pairwise_engagement': read the source and the two rewrites A and B; in the 'choice' cell pick the ONE you would be more likely to click (A or B).</t>
         </is>
@@ -34738,7 +34746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="2" max="2"/>
@@ -34776,22 +34784,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>c3_071</t>
+          <t>c3_070</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>U.S. Congress secures health benefits for coal miners</t>
+          <t>Trump distances himself from remarks on Putin over election meddling</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>What's behind the sudden shift in U.S. Congress's stance on coal miner health benefits?</t>
+          <t>As Trump walks away from controversy over Putin's election influence, where did he draw the line on accountability?</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>What's behind the U.S. Congress's sudden move to secure health benefits for coal miners?</t>
+          <t>What's Behind Trump's Shift on Putin's Election Interference?</t>
         </is>
       </c>
       <c r="E2" s="2" t="n"/>
@@ -34799,22 +34807,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>c3_093</t>
+          <t>c3_085</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Climate change looms large in Obama's final trip to Asia</t>
+          <t>Russia's Putin says Obama administration does not stick to any deals</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>As Obama's Asia trip comes to a close, what's the real agenda behind his climate change focus?</t>
+          <t>"Does Russia's Putin Have a Point: Can Obama Administration Be Trusted to Keep Its Promises?".</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>As Obama's journey to Asia comes to a close, can the world's warming woes be ignored?</t>
+          <t>What's behind Russia's growing frustration with the US over broken promises?</t>
         </is>
       </c>
       <c r="E3" s="2" t="n"/>
@@ -34822,22 +34830,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>c3_051</t>
+          <t>c3_058</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>U.S. Vice President Biden to visit Serbia, Kosovo next week</t>
+          <t>'The Wire' actor Pierce arrested after scuffle over Democratic politics</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>What's behind the U.S. Vice President's surprise trip to Serbia and Kosovo?</t>
+          <t>"Who's Really to Blame: 'The Wire' Actor Pierce's Arrest Raises Questions About Political Passion Getting Out of Hand?".</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>What's behind the sudden diplomatic push: U.S. Vice President Biden to visit Serbia, Kosovo next week?</t>
+          <t>"Who's Behind the Brawl: 'The Wire' Star Pierce Arrested Amid Heated Political Debate?".</t>
         </is>
       </c>
       <c r="E4" s="2" t="n"/>
@@ -34845,22 +34853,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>c3_002</t>
+          <t>c3_065</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook's Sandberg says has no plan to work in government</t>
+          <t>Trump removes Scaramucci as communications director: NYT</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>What's Behind Facebook's Top Executive's Silence on a Potential Government Role?</t>
+          <t>Who's Next in the White House Shake-Up After Scaramucci's Sudden Firing?</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>What's Behind Facebook's Sheryl Sandberg's Decision to Rule Out a Government Role?</t>
+          <t>Trump's Communications Chief Gets the Axe: Can His Replacement Fill the Void Left Behind?</t>
         </is>
       </c>
       <c r="E5" s="2" t="n"/>
@@ -34868,22 +34876,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>c3_024</t>
+          <t>c3_046</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Judge blocks Kansas' attempt to cut Planned Parenthood from Medicaid</t>
+          <t>U.S. Senate approves bill to upgrade airport security</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>What's behind Kansas' sudden move to sever ties with a prominent women's health provider?</t>
+          <t>What's Behind the U.S. Senate's Latest Move to Boost Airport Security?</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>What's behind the sudden halt to Kansas' Medicaid overhaul?</t>
+          <t>As Senate Votes to Bolster Airport Defenses, Are American Travelers Safer Now Than Before?</t>
         </is>
       </c>
       <c r="E6" s="2" t="n"/>
@@ -34891,22 +34899,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>c3_031</t>
+          <t>c3_030</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Clinton scheduled to return to campaign trail on Friday: MSNBC</t>
+          <t>U.S. will not issue some visas in 4 nations in deportation crackdown</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>What's Next for Clinton's Presidential Bid After a Week of Quiet?</t>
+          <t>Who's Being Left Behind in the U.S.'s Latest Deportation Crackdown?</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>What's Next for Clinton's Presidential Bid After a Week of Rest?</t>
+          <t>Whose rights will be left in the balance as U.S. immigration crackdown targets certain countries for visa restrictions?</t>
         </is>
       </c>
       <c r="E7" s="2" t="n"/>
@@ -34914,22 +34922,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>c3_044</t>
+          <t>c3_091</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Trump dips toe into delicate U.S. debt discussion</t>
+          <t>Trump extols corporate profits while seeking corporate tax cut</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>What's driving Trump's sudden interest in the nation's financial future?</t>
+          <t>What's driving the president's push for a corporate tax break?</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>What's behind Trump's cautious wade into America's debt dilemma?</t>
+          <t>As Trump pushes for a corporate tax cut, do profits matter more to big business than to American workers?</t>
         </is>
       </c>
       <c r="E8" s="2" t="n"/>
@@ -34937,22 +34945,22 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>c3_022</t>
+          <t>c3_064</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Exclusive: Trump names career diplomat to head Cuban embassy - sources</t>
+          <t>Trump's Interior Department shortlist vexes employees, green groups</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Who Will Trump Choose to Bridge the Gap Between the US and Cuba?</t>
+          <t>What's behind the secrecy surrounding Trump's Interior Department picks?</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Who Will Trump Choose to Bridge the Gap Between the US and Cuba's Diplomatic Relations? Sources Suggest a Surprise Move is Imminent.</t>
+          <t>Whose interests are Trump's Interior Department prioritizing, and who's left out in the cold?</t>
         </is>
       </c>
       <c r="E9" s="2" t="n"/>
@@ -34960,22 +34968,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>c3_014</t>
+          <t>c3_021</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Mexico president to show 'pragmatism' dealing with Trump</t>
+          <t>New U.S. rule on class actions survives first challenge</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Will Mexico's President Find a Middle Ground with Trump's Unpredictable Style?</t>
+          <t>What's behind the latest court decision to uphold a major shift in U.S. class action law?</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Will Mexico's President Find a Middle Ground with Trump?</t>
+          <t>As a critical test, will court scrutiny spare or scuttle the new U.S. approach to mass lawsuits.</t>
         </is>
       </c>
       <c r="E10" s="2" t="n"/>
@@ -34983,22 +34991,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>c3_012</t>
+          <t>c3_033</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>U.S. lawmakers deadlock on Zika virus funds</t>
+          <t>Meeting between Trump and Japan's Abe has ended: Trump official</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>What's Holding Up the Fight Against Zika? U.S. Lawmakers Stuck in Funding Impasse.</t>
+          <t>What's Behind the Sudden End to Trump's High-Stakes Summit with Japan's Abe?</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>What's Holding Up the Fight Against Zika?</t>
+          <t>After the curtain closes on the private summit: Did Trump and Abe seal a deal or leave the future in limbo?</t>
         </is>
       </c>
       <c r="E11" s="2" t="n"/>
@@ -35006,22 +35014,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>c3_092</t>
+          <t>c3_000</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Senate passes measure that permanently repeals 'Cadillac' tax</t>
+          <t>'Numerous' arrests made during Trump inauguration protests: police</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>What's behind the Senate's sudden shift on a tax that's been a sticking point for years?</t>
+          <t>"Behind the Scenes: What Led to the Wave of Arrests During Trump's Inauguration Protests?".</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>What's behind the Senate's sudden reversal on a tax that's been a thorn in the side of healthcare providers?</t>
+          <t>"Was the force used to quell dissent or protect the crowd during the Trump inauguration protests, as 'numerous' arrests were made by police?".</t>
         </is>
       </c>
       <c r="E12" s="2" t="n"/>
@@ -35029,22 +35037,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>c3_025</t>
+          <t>c3_071</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Trump gets one presidential intelligence briefing a week: sources</t>
+          <t>U.S. Congress secures health benefits for coal miners</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>How often does the President get the latest intel? Just once a week? The truth behind Trump's intelligence briefings.</t>
+          <t>Whose health will be saved by Congress's move to secure benefits for coal miners?</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>How often does the President get the latest intel?</t>
+          <t>What's behind the sudden shift in U.S. Congress's stance on coal miner health benefits?</t>
         </is>
       </c>
       <c r="E13" s="2" t="n"/>
@@ -35052,22 +35060,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>c3_050</t>
+          <t>c3_007</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Trump makes overture to Ryan, while Republicans wrestle with party's future</t>
+          <t>Trump tweet attacking Clinton employs image of Jewish star</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>What's Behind Trump's Unusual Overture to Ryan, as Republicans Grapple with Their Party's Direction?</t>
+          <t>"Did a symbol of resilience and hope become a lightning rod for controversy in Trump's Twitter storm against Clinton?".</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>What's Behind Trump's Unusual Overture to Ryan Amid GOP's Identity Crisis?</t>
+          <t>What's behind Trump's latest tweet targeting Clinton, featuring a symbol with deep historical significance?</t>
         </is>
       </c>
       <c r="E14" s="2" t="n"/>
@@ -35075,22 +35083,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>c3_095</t>
+          <t>c3_089</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>How Egypt's changing culture led one emigre to Trump</t>
+          <t>Seattle mayor drops re-election bid amid sex abuse accusations</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>What drives a former Egyptian expat to find a new home in Trump's America?</t>
+          <t>Seattle Mayor's Sudden Exit Raises Questions About Scandal's Impact on Political Career.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>What drives a person to make a dramatic shift in their life, and what role does cultural evolution play in shaping their decisions?</t>
+          <t>What's behind the sudden departure of Seattle's mayor from the re-election race, amidst allegations of sexual misconduct?</t>
         </is>
       </c>
       <c r="E15" s="2" t="n"/>
@@ -35098,22 +35106,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>c3_088</t>
+          <t>c3_039</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Senate Intelligence committee leaders confirm Kushner testimony</t>
+          <t>Factbox: Trump taps Priebus as chief of staff, weighs other major hires</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>What did Kushner reveal to the Senate Intelligence committee?</t>
+          <t>What's Behind Trump's High-Stakes Staffing Decisions?</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>What did Kushner reveal to the Senate Intelligence committee? Committee leaders confirm his testimony.</t>
+          <t>Whose Hand Will Trump Choose to Guide Him Next: Replacing the Old Guard or Bringing in Fresh Faces?</t>
         </is>
       </c>
       <c r="E16" s="2" t="n"/>
@@ -35121,22 +35129,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>c3_004</t>
+          <t>c3_031</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>U.S. House Republicans to tackle tax plan later this year</t>
+          <t>Clinton scheduled to return to campaign trail on Friday: MSNBC</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>What's on the agenda for U.S. House Republicans as they gear up for a tax plan showdown later this year?</t>
+          <t>Clinton's Comeback?: What Secrets Will She Bring Back to the Campaign Trail on Friday?</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>What's on the agenda for U.S. House Republicans this year: A tax plan in the works?</t>
+          <t>What's Next for Clinton's Presidential Bid After a Week of Quiet?</t>
         </is>
       </c>
       <c r="E17" s="2" t="n"/>
@@ -35144,22 +35152,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>c3_000</t>
+          <t>c3_053</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>'Numerous' arrests made during Trump inauguration protests: police</t>
+          <t>Justice Department antitrust nominee Makan Delrahim's hearing delayed</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>"Behind the Scenes: What Led to the Wave of Arrests During Trump's Inauguration Protests?".</t>
+          <t>What's Behind the Delay of Makan Delrahim's Justice Department Antitrust Nomination Hearing?</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>"Was the force used to quell dissent or protect the crowd during the Trump inauguration protests, as 'numerous' arrests were made by police?".</t>
+          <t>When Will Answers Emerge Delay in Justice Department's Antitrust Nominee Hearing Sparks Questions.</t>
         </is>
       </c>
       <c r="E18" s="2" t="n"/>
@@ -35167,22 +35175,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>c3_017</t>
+          <t>c3_051</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>U.S. coal stocks fall; exit from climate deal may hurt, not help</t>
+          <t>U.S. Vice President Biden to visit Serbia, Kosovo next week</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Will a sudden shift in climate policy send U.S. coal stocks plummeting?</t>
+          <t>What's behind the sudden diplomatic push: U.S. Vice President Biden to visit Serbia, Kosovo next week?</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Will a hasty retreat from climate commitments ignite a coal crisis in the U.S.?</t>
+          <t>"Will a high-stakes US diplomatic trip to Serbia and Kosovo next week bring lasting peace to the region?".</t>
         </is>
       </c>
       <c r="E19" s="2" t="n"/>
@@ -35190,22 +35198,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>c3_028</t>
+          <t>c3_004</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Rights advocates slam Trump plans on Muslim immigrants, refugees</t>
+          <t>U.S. House Republicans to tackle tax plan later this year</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>What's Behind the Controversy Over Trump's Latest Immigration Policy Shift?</t>
+          <t>As lawmakers gear up for a busy legislative season, will tax reform take center stage in the U.S. House later this year?</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>What's Behind the Backlash Against Trump's New Immigration Strategy?</t>
+          <t>What's on the agenda for U.S. House Republicans this year: A tax plan in the works?</t>
         </is>
       </c>
       <c r="E20" s="2" t="n"/>
@@ -35213,22 +35221,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>c3_045</t>
+          <t>c3_062</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Trump tax plan expends recession-fighting U.S. business tax break</t>
+          <t>Trump and Obama set campaign rancor aside with White House meeting</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Will a key recession-fighting tax break be spared as part of Trump's economic overhaul?</t>
+          <t>What's Behind the Unlikely Truce Between Trump and Obama?</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Will a key recession-fighting tool be sacrificed in the name of tax reform? The fate of a crucial U.S. business tax break hangs in the balance.</t>
+          <t>Trump and Obama Make History with Surprise Encounter Amid Election Season Tensions.</t>
         </is>
       </c>
       <c r="E21" s="2" t="n"/>
@@ -35236,22 +35244,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>c3_083</t>
+          <t>c3_097</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Argentine TV ad mocks Trump to promote soccer tournament</t>
+          <t>As debt limit looms, House leaders eye bipartisan deal</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>What's behind the cheeky jab at the White House in Argentina's latest TV ad?</t>
+          <t>As debt limit approaches, are House leaders secretly cooking up a compromise that could surprise everyone?</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>What's behind the cheeky jab at the White House in a new Argentine TV ad?</t>
+          <t>Will House Leaders Find a Last-Minute Solution to Avoid a Fiscal Showdown?</t>
         </is>
       </c>
       <c r="E22" s="2" t="n"/>
@@ -35259,22 +35267,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>c3_091</t>
+          <t>c3_059</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Trump extols corporate profits while seeking corporate tax cut</t>
+          <t>White House says rollback of Obamacare must be part of short-term fix</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>What's driving the president's push for a corporate tax break?</t>
+          <t>What's the Price of a Quick Obamacare Fix?</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>What's driving Trump's push for a corporate tax cut, despite soaring profits?</t>
+          <t>As lawmakers scramble for a solution, will Obamacare rollback be a key piece of the pie to stabilize healthcare costs in the short term?</t>
         </is>
       </c>
       <c r="E23" s="2" t="n"/>
@@ -35282,22 +35290,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>c3_008</t>
+          <t>c3_056</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Obama to press Trump to preserve Cuba detente: White House</t>
+          <t>Senator Warren seeks investigation of insurers over retirement rule</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Will Trump's Cuba Policy Stay on Course?</t>
+          <t>Senator Warren Calls for a Probe into Insurers' Retirement Rule Tactics Amid Fears of Financial Fallout.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Will Trump's Cuba Policy Stay the Course Under Pressure from Obama's Legacy? The White House Weighs In.</t>
+          <t>What's Behind Senator Warren's Call for a Probe into Insurers' Retirement Rule?</t>
         </is>
       </c>
       <c r="E24" s="2" t="n"/>
@@ -35305,22 +35313,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>c3_027</t>
+          <t>c3_078</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>U.S. House clears path for tax bill with budget approval</t>
+          <t>Obama says EU and U.S. must move forward with TTIP</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>What's the Next Move for Tax Reform After Budget Breakthrough?</t>
+          <t>What's Holding Up the EU-US Trade Deal?</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>What's Next for Tax Reform as Budget Hurdle is Cleared?</t>
+          <t>As TTIP Talks Stall, Are Leaders Ready to Break Impasse and Seal Deal with EU and U.S. Together?</t>
         </is>
       </c>
       <c r="E25" s="2" t="n"/>
@@ -35328,22 +35336,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>c3_075</t>
+          <t>c3_080</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Factbox: Clean energy faces vote in four state ballot initiatives</t>
+          <t>Figures show Trump spent $66 million of his own cash on election campaign</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>What's at Stake: Clean Energy's Future Hangs in the Balance as Four States Prepare to Cast Their Votes.</t>
+          <t>What's behind the staggering $66 million personal investment in Trump's election bid?</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>What's at Stake: Will Voters Choose a Cleaner Future for Four States?</t>
+          <t>Just $66 million of your own cash: Did it buy the presidency for Trump?</t>
         </is>
       </c>
       <c r="E26" s="2" t="n"/>
@@ -35351,22 +35359,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>c3_097</t>
+          <t>c3_018</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>As debt limit looms, House leaders eye bipartisan deal</t>
+          <t>Trump says working on welfare reform proposals</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Will House Leaders Find a Last-Minute Solution to Avoid a Fiscal Showdown?</t>
+          <t>What's Next for Welfare Reform: Trump's Plans Take Shape.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Will House Leaders Find a Last-Minute Solution to Avoid a Fiscal Showdown? As Debt Limit Looms, Can They Strike a Bipartisan Bargain?</t>
+          <t>As Trump Looks Ahead, What Shape Will Welfare Overhaul Take?</t>
         </is>
       </c>
       <c r="E27" s="2" t="n"/>
@@ -35374,22 +35382,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>c3_074</t>
+          <t>c3_077</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Putin says he doesn't know who hacked U.S. Democratic Party: Bloomberg</t>
+          <t>Italian prime minister to meet Trump in U.S. on April 20: diplomatic sources</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Who's behind the U.S. Democratic Party's cyber woes, and is Putin in the dark?</t>
+          <t>Whose diplomatic dance will dominate the White House stage on April 20? Italian prime minister's secret meeting with Trump sends intrigue soaring.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Who's behind the alleged breach of U.S. Democratic Party data, according to Putin's latest statement?</t>
+          <t>What's on the agenda for the Italian prime minister's high-stakes meeting with Trump on April 20?</t>
         </is>
       </c>
       <c r="E28" s="2" t="n"/>
@@ -35397,22 +35405,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>c3_030</t>
+          <t>c3_050</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>U.S. will not issue some visas in 4 nations in deportation crackdown</t>
+          <t>Trump makes overture to Ryan, while Republicans wrestle with party's future</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Who's Being Left Behind in the U.S.'s Latest Deportation Crackdown?</t>
+          <t>What's Behind Trump's Unusual Overture to Ryan Amid GOP's Identity Crisis?</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Who's Being Left Behind in the U.S.'s Latest Deportation Crackdown? Visa Holders in 4 Nations Will Be Denied Entry.</t>
+          <t>As Trump reaches out to Ryan, what lies ahead for the GOP's uncertain trajectory?</t>
         </is>
       </c>
       <c r="E29" s="2" t="n"/>
@@ -35420,22 +35428,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>c3_019</t>
+          <t>c3_037</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Clinton heavily favored to win Electoral College: poll</t>
+          <t>Trump aide says no decision on Clinton prosecutor, now focused on unity</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Who's Poised to Sweep the Electoral College: A New Poll Reveals the Surprising Favorite.</t>
+          <t>As Unity Efforts Gain Steam, Is a Clinton Prosecutor in the Rearview Mirror for Trump's Team at Last?</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Who's Poised to Sweep the Electoral College: A New Poll Reveals a Surprising Favorite.</t>
+          <t>What's Next for the White House: Unity or Justice?</t>
         </is>
       </c>
       <c r="E30" s="2" t="n"/>
@@ -35443,22 +35451,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>c3_064</t>
+          <t>c3_020</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Trump's Interior Department shortlist vexes employees, green groups</t>
+          <t>Pennsylvania mayors charged in pay-to-play corruption case</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>What's behind the secrecy surrounding Trump's Interior Department picks?</t>
+          <t>Who's Behind the Cash-For-Favors Scandal Rocking Pennsylvania's Mayoral Offices?</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>What's behind the Interior Department's latest personnel puzzle, leaving employees and environmental advocates scratching their heads?</t>
+          <t>Whose Power Brokers Behind Bars in Corruption Crackdown Have Been Caught Red-handed in Pennsylvania's Political Underbelly?</t>
         </is>
       </c>
       <c r="E31" s="2" t="n"/>
@@ -35466,22 +35474,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>c3_065</t>
+          <t>c3_025</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Trump removes Scaramucci as communications director: NYT</t>
+          <t>Trump gets one presidential intelligence briefing a week: sources</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Who's Next in the White House Shuffle After Scaramucci's Sudden Exit? Trump's Communications Director Out.</t>
+          <t>Just one secret briefing a week: does it give Trump enough intel to lead effectively?</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Who's Next in the White House Shake-Up After Scaramucci's Sudden Firing?</t>
+          <t>How often does the President get the latest intel?</t>
         </is>
       </c>
       <c r="E32" s="2" t="n"/>
@@ -35489,22 +35497,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>c3_096</t>
+          <t>c3_045</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Trump, Lockheed Martin CEO to meet on Friday: transition official</t>
+          <t>Trump tax plan expends recession-fighting U.S. business tax break</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>What's on the agenda for Trump's meeting with Lockheed Martin's top brass on Friday?</t>
+          <t>Will a key recession-fighting tax break be spared as part of Trump's economic overhaul?</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>What's on the agenda for Trump's meeting with Lockheed Martin's top boss on Friday?</t>
+          <t>As recession looms, is America's business tax shield on shaky ground, courtesy of Trump's tax plan rethink?</t>
         </is>
       </c>
       <c r="E33" s="2" t="n"/>
@@ -35512,22 +35520,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>c3_086</t>
+          <t>c3_024</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Obama's prisoner clemency plan faltering as cases pile up</t>
+          <t>Judge blocks Kansas' attempt to cut Planned Parenthood from Medicaid</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>As Obama's pardon pipeline slows to a trickle, will justice be delayed for those waiting in the wings?</t>
+          <t>"Can Medicaid funding for reproductive health services survive legal challenges in Kansas, or will access be restricted by court intervention?".</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>As Obama's deadline looms, a backlog of hopefuls threatens to derail his bid to set prisoners free.</t>
+          <t>What's behind the sudden halt to Kansas' Medicaid overhaul?</t>
         </is>
       </c>
       <c r="E34" s="2" t="n"/>
@@ -35535,22 +35543,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>c3_078</t>
+          <t>c3_068</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Obama says EU and U.S. must move forward with TTIP</t>
+          <t>Trump: military solutions 'locked and loaded' against North Korea threat</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>What's Holding Up the EU-US Trade Deal? Obama Calls for Progress on Key Agreement.</t>
+          <t>As tensions simmer, will Trump's stern ultimatum appease Pyongyang, or risk sparking conflict in East Asia?</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>What's Holding Up the EU-US Trade Deal?</t>
+          <t>What's Behind the President's Threats to Take Action Against North Korea?</t>
         </is>
       </c>
       <c r="E35" s="2" t="n"/>
@@ -35558,22 +35566,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>c3_082</t>
+          <t>c3_009</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>White House names retired Air Force general as first cyber security chief</t>
+          <t>Republicans grapple with whether to back Trump for White House</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Who Will Lead the Charge in Protecting the Nation's Digital Frontlines?</t>
+          <t>As Trump's fate in the White House hangs in the balance, can GOP loyalists square the circle on supporting their standard-bearer or chart a new course?</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Who Will Lead the Charge in Protecting the Nation's Digital Frontlines as White House Taps Retired Air Force General for Top Cyber Security Post?</t>
+          <t>What's the Future of Trump's Presidential Ambitions for the GOP?</t>
         </is>
       </c>
       <c r="E36" s="2" t="n"/>
@@ -35581,22 +35589,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>c3_060</t>
+          <t>c3_055</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Obama, Republican leaders seek elusive common ground in White House meeting</t>
+          <t>LinkedIn's Hoffman: Trump presidency would be 'terrifying' for policy</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>What's the Secret to Bridging the Divide: Obama and GOP Leaders Meet Behind Closed Doors.</t>
+          <t>As Trump Takes Office: Will America Sleep Easy Under a New Era of Uncertainty?</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>What's the Secret to Bridging the Divide? Obama and GOP Leaders Meet Behind Closed Doors.</t>
+          <t>What would a Trump presidency mean for LinkedIn's policy landscape?</t>
         </is>
       </c>
       <c r="E37" s="2" t="n"/>
@@ -35604,22 +35612,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>c3_066</t>
+          <t>c3_017</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Marco Rubio emerges as champion of battered Republican establishment</t>
+          <t>U.S. coal stocks fall; exit from climate deal may hurt, not help</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Who's the unlikely hero rallying the Republican faithful back to the fold? Marco Rubio's sudden surge sparks questions about the party's future.</t>
+          <t>Will a hasty retreat from climate commitments ignite a coal crisis in the U.S.?</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Who's the unlikely hero rallying the Republican faithful?</t>
+          <t>As Climate Deal's Fate Lies in Balance: Will U.S. Coal Industry Pay the Price for Its Departure from Global Accord?</t>
         </is>
       </c>
       <c r="E38" s="2" t="n"/>
@@ -35627,22 +35635,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>c3_077</t>
+          <t>c3_013</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Italian prime minister to meet Trump in U.S. on April 20: diplomatic sources</t>
+          <t>Factbox: Highlights of Trump's calls with leaders of Mexico, Australia</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>What's on the agenda for the Italian prime minister's high-stakes meeting with Trump on April 20?</t>
+          <t>Whispers from the White House: Did Trump's diplomatic outreach yield more than meets the eye in conversations with Mexico and Australia?</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>What's on the agenda when Italy's PM meets Trump in the US on April 20?</t>
+          <t>What secrets did Trump reveal in his phone calls with Mexico and Australia?</t>
         </is>
       </c>
       <c r="E39" s="2" t="n"/>
@@ -35650,22 +35658,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>c3_073</t>
+          <t>c3_057</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Trump considering Mitt Romney for secretary of state: NBC News</t>
+          <t>Trump says he will order 'safe zones' for Syria</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Who's Next in Line for Trump's Top Diplomatic Post?</t>
+          <t>What's Behind Trump's Promise to Create 'Safe Havens' in Syria?</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Who's Next in Line for Trump's Top Diplomatic Post? Could a Familiar Face Get the Job?</t>
+          <t>As Trump prepares to act in Syria, will fragile regions of the war-torn country become the next focal point of international attention?</t>
         </is>
       </c>
       <c r="E40" s="2" t="n"/>
@@ -35673,22 +35681,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>c3_054</t>
+          <t>c3_098</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Should I stay or should I go? U.S. civil servants gird for Trump</t>
+          <t>Trump: 'most likely' would choose a Supreme Court nominee from list</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>As the clock ticks, what's next for America's public servants in the face of uncertainty?</t>
+          <t>Who's on the shortlist for Trump's next Supreme Court pick?</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>As uncertainty looms, are U.S. civil servants preparing for a sudden departure or a prolonged stay under Trump's leadership?</t>
+          <t>"Will the President Opt for a Pre-Vetted Justice or Take a Gamble on a New Nominee?".</t>
         </is>
       </c>
       <c r="E41" s="2" t="n"/>
@@ -35696,22 +35704,22 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>c3_037</t>
+          <t>c3_028</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Trump aide says no decision on Clinton prosecutor, now focused on unity</t>
+          <t>Rights advocates slam Trump plans on Muslim immigrants, refugees</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>What's Next for the White House: Unity or Justice?</t>
+          <t>What's Behind the Controversy Over Trump's Latest Immigration Policy Shift?</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>What's Next for the White House: Unity or Justice for Clinton?</t>
+          <t>As Trump's stance on Muslim immigrants and refugees stirs divided debate, who benefits from his proposed measures and who pays the price?</t>
         </is>
       </c>
       <c r="E42" s="2" t="n"/>
@@ -35719,22 +35727,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>c3_079</t>
+          <t>c3_095</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Oil mogul Hamm tops Trump list for U.S. energy secretary: sources</t>
+          <t>How Egypt's changing culture led one emigre to Trump</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Who's the top pick to shape America's energy future, according to Trump's inner circle?</t>
+          <t>Whose journey from Egypt to Trump was driven by shifting values at home?</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Who's the top pick to shape America's energy future, according to insiders close to the White House?</t>
+          <t>What drives a person to make a dramatic shift in their life, and what role does cultural evolution play in shaping their decisions?</t>
         </is>
       </c>
       <c r="E43" s="2" t="n"/>
@@ -35742,22 +35750,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>c3_010</t>
+          <t>c3_090</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Russia U.N. envoy says U.S. sanctions will not change Moscow</t>
+          <t>Path cleared for Congress to consider U.S. arms sale to Riyadh: State Department</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Will Russia's Stance on U.S. Sanctions Remain Unwavering? What's Behind Moscow's Confidence?</t>
+          <t>What's Next for U.S. Arms Deal with Riyadh as Path Cleared for Congressional Review?</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Will Russia's Stance on U.S. Sanctions Remain Unwavering?</t>
+          <t>As a critical juncture approaches, will Congress seize the opportunity to greenlight a major U.S. arms deal with Saudi Arabia, or will concerns hold them back?</t>
         </is>
       </c>
       <c r="E44" s="2" t="n"/>
@@ -35765,22 +35773,22 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>c3_055</t>
+          <t>c3_040</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>LinkedIn's Hoffman: Trump presidency would be 'terrifying' for policy</t>
+          <t>Factbox: Trump on Twitter (Sept 26) - NFL ratings, Nikki Haley, Spain</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>What would a Trump presidency mean for LinkedIn's policy landscape?</t>
+          <t>"Did Trump's Sept 26 Tweets Send NFL Ratings and Nikki Haley's Profile Skyrocketing... or Sinking in Spain?".</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>What would a Trump presidency mean for LinkedIn's policy landscape? LinkedIn's Hoffman speaks out on the potential impact.</t>
+          <t>What's Behind Trump's Social Media Rant About the NFL and International Affairs?</t>
         </is>
       </c>
       <c r="E45" s="2" t="n"/>
@@ -35788,22 +35796,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>c3_006</t>
+          <t>c3_035</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Hurricane Matthew toll in Haiti rises to 1,000, dead buried in mass graves</t>
+          <t>Trump strategy document says Russia meddles in domestic affairs worldwide</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>As Haiti's Death Toll Surpasses 1,000, a Grim Reality Emerges.</t>
+          <t>As global tensions simmer, does Moscow secretly manipulate internal politics across borders, according to a confidential Trump administration report?</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>As the storm's devastating aftermath unfolds, can Haiti's true death toll be hidden forever?</t>
+          <t>What's behind the global reach of Russia's alleged meddling in domestic affairs?</t>
         </is>
       </c>
       <c r="E46" s="2" t="n"/>
@@ -35811,22 +35819,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>c3_058</t>
+          <t>c3_074</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>'The Wire' actor Pierce arrested after scuffle over Democratic politics</t>
+          <t>Putin says he doesn't know who hacked U.S. Democratic Party: Bloomberg</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>"Who's Behind the Brawl: 'The Wire' Star Pierce Arrested Amid Heated Political Debate?".</t>
+          <t>Who's behind the alleged breach of U.S. Democratic Party data, according to Putin's latest statement?</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>"Who's Really Behind the Latest Celebrity Arrest: A Scuffle Over Politics or Something More?".</t>
+          <t>Whose hand may have struck fear into the heart of U.S. Democratic Party emails? Putin is tight-lipped.</t>
         </is>
       </c>
       <c r="E47" s="2" t="n"/>
@@ -35834,22 +35842,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>c3_059</t>
+          <t>c3_047</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>White House says rollback of Obamacare must be part of short-term fix</t>
+          <t>Trump to meet with airline CEOs on Thursday: White House</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>What's the Price of a Quick Obamacare Fix?</t>
+          <t>Thursday's White House Summit: Are Airline Passengers' Worries About to Take Flight with Trump's Meeting with Industry Leaders?</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>What's the Price of a Quick Obamacare Fix: Rollback a Must?</t>
+          <t>What's on the agenda for Trump's meeting with airline CEOs on Thursday?</t>
         </is>
       </c>
       <c r="E48" s="2" t="n"/>
@@ -35857,22 +35865,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>c3_029</t>
+          <t>c3_096</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Exclusive: Trump boosts disaster aid for Puerto Rico rebuild</t>
+          <t>Trump, Lockheed Martin CEO to meet on Friday: transition official</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>What's Behind Trump's Sudden Shift in Disaster Relief for Puerto Rico?</t>
+          <t>"Who's behind the closed-door talks as Trump gears up to shape defense landscape with Lockheed Martin CEO this Friday?".</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>What's Behind Trump's Sudden Shift in Disaster Relief for Puerto Rico's Reconstruction Efforts?</t>
+          <t>What's on the agenda for Trump's meeting with Lockheed Martin's top boss on Friday?</t>
         </is>
       </c>
       <c r="E49" s="2" t="n"/>
@@ -35880,22 +35888,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>c3_098</t>
+          <t>c3_092</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Trump: 'most likely' would choose a Supreme Court nominee from list</t>
+          <t>Senate passes measure that permanently repeals 'Cadillac' tax</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Who's on the shortlist for the next Supreme Court justice, and what does it mean for the future of the court?</t>
+          <t>"Will the End of the 'Cadillac' Tax Mark a New Era in Healthcare Funding?".</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Who's on the shortlist for Trump's next Supreme Court pick?</t>
+          <t>What's behind the Senate's sudden shift on a tax that's been a sticking point for years?</t>
         </is>
       </c>
       <c r="E50" s="2" t="n"/>
@@ -35903,22 +35911,22 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>c3_061</t>
+          <t>c3_011</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Michigan governor names panel to fix Flint's contaminated water system</t>
+          <t>From Wall Street to Wisconsin, brokers cheer Trump's order</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>What's the Plan to Finally Fix Flint's Toxic Water Crisis?</t>
+          <t>What's behind the sudden surge of optimism on Wall Street and in the heartland?</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>What's Behind the Governor's Plan to Revamp Flint's Toxic Water Crisis?</t>
+          <t>As Trump's decree sends ripples from Manhattan to Madison, will big finance's enthusiasm translate to Main Street prosperity?</t>
         </is>
       </c>
       <c r="E51" s="2" t="n"/>
@@ -35926,22 +35934,22 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>c3_047</t>
+          <t>c3_079</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Trump to meet with airline CEOs on Thursday: White House</t>
+          <t>Oil mogul Hamm tops Trump list for U.S. energy secretary: sources</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>What's on the agenda when Trump sits down with airline bosses on Thursday? White House reveals all.</t>
+          <t>Whose Surging Rise to Power Will Shape America's Energy Future: Secrets of the Trump Shortlist Reveal Few Surprises.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>What's on the agenda for Trump's meeting with airline CEOs on Thursday?</t>
+          <t>Who's the top pick to shape America's energy future, according to Trump's inner circle?</t>
         </is>
       </c>
       <c r="E52" s="2" t="n"/>
@@ -35949,22 +35957,22 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>c3_067</t>
+          <t>c3_003</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>U.S. Democrats' infighting over trade pact puts Clinton in middle</t>
+          <t>Justice Department weighs changes to Obama-era financial task force</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>As tensions simmer among U.S. Democrats, who will ultimately sway Clinton's stance on a contentious trade agreement?</t>
+          <t>What's Behind the Justice Department's Reevaluation of a Key Financial Oversight Tool?</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>As tensions simmer among U.S. Democrats over a contentious trade agreement, can Hillary Clinton's diplomatic skills help broker a compromise?</t>
+          <t>As Justice Department Weighs Shifts to Financial Task Force, Are the Foundations of Consumer Protection at Risk of Erosion?</t>
         </is>
       </c>
       <c r="E53" s="2" t="n"/>
@@ -35972,22 +35980,22 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>c3_069</t>
+          <t>c3_008</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>'You're wrong', Tillerson says of reports he will be fired</t>
+          <t>Obama to press Trump to preserve Cuba detente: White House</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>"Is the Rumored Shake-Up at the Top About to Get a Reality Check?".</t>
+          <t>Will Trump Listen to Obama's Plea to Keep Cuba Relations on Course? White House Insights Suggest a Shift Ahead.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>"Who's next on the chopping block? Tillerson's blunt denial sparks questions about his future".</t>
+          <t>Will Trump's Cuba Policy Stay on Course?</t>
         </is>
       </c>
       <c r="E54" s="2" t="n"/>
@@ -35995,22 +36003,22 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>c3_094</t>
+          <t>c3_054</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Trump blasts former Scottish leader as war of words grows</t>
+          <t>Should I stay or should I go? U.S. civil servants gird for Trump</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>As tensions escalate, what sparks the fiery rhetoric between Trump and a former Scottish leader?</t>
+          <t>As uncertainty looms, will loyal public workers stick or split with a president who's still got a few cards up his sleeve?</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>As tensions escalate, what's behind the escalating rhetoric between Trump and a former Scottish leader?</t>
+          <t>As the clock ticks, what's next for America's public servants in the face of uncertainty?</t>
         </is>
       </c>
       <c r="E55" s="2" t="n"/>
@@ -36018,22 +36026,22 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>c3_034</t>
+          <t>c3_082</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Senate banking panel approves Szubin for key sanctions post</t>
+          <t>White House names retired Air Force general as first cyber security chief</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Who Will Shape the Future of Global Finance: Senate Panel Greenlights Key Appointment?</t>
+          <t>"Who will lead the quest to protect America's digital defenses, now that a seasoned warrior from the skies has taken the helm at the White House?".</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Who Will Lead the Charge in Enforcing Economic Sanctions After Senate Panel Gives Key Nod?</t>
+          <t>Who Will Lead the Charge in Protecting the Nation's Digital Frontlines?</t>
         </is>
       </c>
       <c r="E56" s="2" t="n"/>
@@ -36041,22 +36049,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>c3_007</t>
+          <t>c3_010</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Trump tweet attacking Clinton employs image of Jewish star</t>
+          <t>Russia U.N. envoy says U.S. sanctions will not change Moscow</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>What sparks controversy in Trump's latest tweet: A symbol with a complex history takes center stage.</t>
+          <t>Will Russia's Stance on U.S. Sanctions Remain Unwavering?</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>What's behind Trump's latest tweet targeting Clinton, featuring a symbol with deep historical significance?</t>
+          <t>As Russia's stance at the UN remains firm: Will US sanctions be enough to shift Moscow's course?</t>
         </is>
       </c>
       <c r="E57" s="2" t="n"/>
@@ -36064,22 +36072,22 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>c3_087</t>
+          <t>c3_041</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>California bill to fight fashion models' eating disorders advances</t>
+          <t>White House continues to cooperate with special counsel -official</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>As California lawmakers take a step forward in addressing a hidden health crisis, can the fashion industry's influence be far behind in the fight against eating disorders?</t>
+          <t>What's Behind the White House's Ongoing Cooperation with the Special Counsel?</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>As California lawmakers take a step forward, what's driving the push to protect models from the dark side of the fashion industry?</t>
+          <t>As Questions Linger, White House Cooperation with Investigators Remains Unwavering.</t>
         </is>
       </c>
       <c r="E58" s="2" t="n"/>
@@ -36087,22 +36095,22 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>c3_042</t>
+          <t>c3_022</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Trump wants ex-Goldman partner Mnuchin to run U.S. Treasury: Fox Business</t>
+          <t>Exclusive: Trump names career diplomat to head Cuban embassy - sources</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Who will Trump tap to steer the nation's finances, and what does it say about his economic priorities?</t>
+          <t>Who Will Trump Choose to Bridge the Gap Between the US and Cuba?</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Who will Trump tap as his next Treasury Secretary and why is a former Goldman Sachs executive in the running? Fox Business reports.</t>
+          <t>Whose diplomatic expertise will be put to the test in Havana? Sources say Trump has chosen a career diplomat to lead US efforts in Cuba.</t>
         </is>
       </c>
       <c r="E59" s="2" t="n"/>
@@ -36110,29 +36118,972 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
+          <t>c3_048</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Trump to keep Manhattan federal prosecutor Bharara in post</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>"Will Trump's Move to Keep Manhattan's Top Prosecutor Send a Message to the Justice System?".</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>What's Behind Trump's Decision to Keep Manhattan's Top Prosecutor on Board?</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>c3_066</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Marco Rubio emerges as champion of battered Republican establishment</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Who's the unlikely hero rallying the Republican faithful?</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Whose corner is Marco Rubio fighting for in Republican politics' latest power shift?</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>c3_088</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Senate Intelligence committee leaders confirm Kushner testimony</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>What did Kushner reveal to the Senate Intelligence committee?</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Kushner's Testimony Put Under Senate Intelligence Committee's Spotlight? Will Revelations Shed New Light on His Role?</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>c3_001</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>U.S. lawmakers ask Trump to turn over any Comey tapes</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>"Did Trump Record His Conversations with Comey - and Will He Share Them with Congress Now?".</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>What's Behind the President's Silence on the Comey Conversations?</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>c3_081</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>How to rebuild Puerto Rico: Rubio asks Trump to call in experts</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>As Puerto Rico's Future Hangs in the Balance, Can Trump's Team Deliver the Expertise Needed to Rebuild the Island?</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>What's the secret to Puerto Rico's recovery? Rubio urges Trump to tap into expertise.</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>c3_006</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Hurricane Matthew toll in Haiti rises to 1,000, dead buried in mass graves</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>As Haiti's Death Toll Passes 1,000: Can Mass Graves Provide Closure for Families of Victims of Hurricane Matthew's Devastation?</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>As Haiti's Death Toll Surpasses 1,000, a Grim Reality Emerges.</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>c3_044</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Trump dips toe into delicate U.S. debt discussion</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Trump wades into the complicated waters of America's debt future.</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>What's driving Trump's sudden interest in the nation's financial future?</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>c3_094</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Trump blasts former Scottish leader as war of words grows</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>As tensions escalate, what's behind the escalating rhetoric between Trump and a former Scottish leader?</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>As tensions simmer, did a scorching rebuke from Trump mark a low point in a simmering feud with a former Scottish leader?</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>c3_086</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Obama's prisoner clemency plan faltering as cases pile up</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>As Obama's pardon pipeline slows to a trickle, will justice be delayed for thousands of inmates on death row?</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>As Obama's deadline looms, a backlog of hopefuls threatens to derail his bid to set prisoners free.</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>c3_052</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Senate votes to confirm Gottlieb as head of FDA</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Will Gottlieb's Appointment as FDA Chief Bring a New Era of Regulation?</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Whose Health Will FDA's New Leader Prioritize First? Senate Votes Yes to Confirmation.</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>c3_072</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Supreme Court nominee to submit questionnaire to lawmakers</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>As Supreme Court Nominee Faces Questions from Lawmakers What Secrets Will Be Revealed?</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>What's Behind the Supreme Court Nominee's Answer Sheet for Lawmakers?</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>c3_019</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Clinton heavily favored to win Electoral College: poll</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>As Election Day Looms, Are Clinton's Chances of Securing the Electoral College Too Strong to Overcome?</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Who's Poised to Sweep the Electoral College: A New Poll Reveals the Surprising Favorite.</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>c3_038</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Obama says world must unite to defeat terrorism</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Can the world's leaders find common ground to combat a growing threat?</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>As global threats loom large, are nations strong enough to stand united against the forces of destruction?</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>c3_087</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>California bill to fight fashion models' eating disorders advances</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>As California lawmakers take a step forward, what's driving the push to protect models from the dark side of the fashion industry?</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>As California lawmakers move closer to passing a bill to combat eating disorders among fashion models, can a single industry's influence on body image be too great?</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>c3_014</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Mexico president to show 'pragmatism' dealing with Trump</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Will Mexico's President Find a Middle Ground with Trump?</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>As Mexico's leader prepares to negotiate with Trump: Will pragmatism be enough to bridge the divide?</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>c3_005</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>California Senate passes gun control package</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>What's behind the California Senate's decisive move on gun control?</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>California Senate takes decisive step towards stricter gun laws.</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>c3_027</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>U.S. House clears path for tax bill with budget approval</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>What's the Next Move for Tax Reform After Budget Breakthrough?</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>As lawmakers clear hurdles, is a tax overhaul on track for swift passage after budget deal is sealed in the U.S. House today?</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>c3_049</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Trump administration sides with employers in Supreme Court labor case</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Whose interests will tip the balance in the Supreme Court's high-stakes labor showdown?</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>What does the Trump administration's stance on labor rights reveal about its priorities?</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>c3_075</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Factbox: Clean energy faces vote in four state ballot initiatives</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>What's at Stake: Clean Energy's Future Hangs in the Balance as Four States Prepare to Cast Their Votes.</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Whose Future Will Be Powered by Clean Energy Come Election Day in Four States?</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>c3_036</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>U.S. Republican Rand Paul suspends 2016 White House campaign</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>What's Behind Rand Paul's Sudden Decision to Halt His Presidential Bid?</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Rand Paul's Presidential Bid Takes an Unexpected Turn: What's Behind the Sudden Halt?</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>c3_083</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Argentine TV ad mocks Trump to promote soccer tournament</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>What's behind the cheeky jab at the White House in a new Argentine TV ad?</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>"Is satire the new way to score big with Argentine audiences?".</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>c3_026</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Factbox: Trump to meet with U.S. House Speaker Ryan, U.S. Senator Manchin</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Factbox: What's on the Agenda for Trump's High-Stakes Meeting with Ryan and Manchin?</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>What's on the Agenda for Trump's High-Stakes Meetings with Top Lawmakers?</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>c3_042</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Trump wants ex-Goldman partner Mnuchin to run U.S. Treasury: Fox Business</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Who will Trump tap to steer the nation's finances, and what does it say about his economic priorities?</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>"Who will Trump choose to steer the U.S. economy and how will it impact America's financial future, now that he's eyeing a familiar face for the Treasury post?".</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>c3_016</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Democratic candidate for Senate concedes runoff in Louisiana</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Will Louisiana's Democratic Hopes Fade Away with Senate Runoff Concession?</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>After a Tight Battle, Is the Democratic Senate Bid in Louisiana Hitting Roadblock 30 Feet from Victory Line?</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
           <t>c3_076</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B84" t="inlineStr">
         <is>
           <t>U.S. conservatives cancel invitation for firebrand commentator</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C84" t="inlineStr">
         <is>
           <t>Who's Behind the Last-Minute Cancellation of a Firebrand's U.S. Appearance?</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Who's Behind the Sudden U-Turn: U.S. Conservatives Withdraw Invitation to Prolific Voice?</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="n"/>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>"Who's Off the Guest List? Why Did U.S. Conservatives Suddenly Cut Ties with a Controversial Voice?".</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>c3_069</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>'You're wrong', Tillerson says of reports he will be fired</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>"Tillerson's Tone Turns Tense as Denial of Departure Rumors Spark Questions: Am I Next Out the Door?".</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>"Who's next on the chopping block? Tillerson's blunt denial sparks questions about his future".</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>c3_073</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Trump considering Mitt Romney for secretary of state: NBC News</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Who's Next in Line for Trump's Top Diplomatic Post?</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Whose diplomacy expertise will Trump tap for his cabinet's top post, according to NBC News reports?</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>c3_029</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Exclusive: Trump boosts disaster aid for Puerto Rico rebuild</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>What's Behind Trump's Sudden Shift in Disaster Relief for Puerto Rico?</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>As Puerto Rico Looks Beyond Devastation, Will Trump's Boosted Aid Prove Sufficient for Rebuilding Efforts.</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>c3_034</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Senate banking panel approves Szubin for key sanctions post</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>"Who will wield the power to shape US economic policy with this latest Senate appointment?".</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Who Will Lead the Charge in Enforcing Economic Sanctions After Senate Panel Gives Key Nod?</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>c3_067</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>U.S. Democrats' infighting over trade pact puts Clinton in middle</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>As tensions simmer among U.S. Democrats over a high-stakes trade agreement, can party insiders trust Hillary Clinton to navigate the treacherous waters of compromise?</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>As tensions simmer among U.S. Democrats, who will ultimately sway Clinton's stance on a contentious trade agreement?</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>c3_084</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>U.S. says holds Myanmar military leaders accountable in Rohingya crisis</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>What's behind the U.S. decision to hold Myanmar's military leaders accountable for the Rohingya crisis?</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>As Myanmar's Rohingya crisis deepens, can accountability for military leaders really be a game-changer for the region's future?</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>c3_093</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Climate change looms large in Obama's final trip to Asia</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>As Obama's Asia journey concludes, will climate's shadow follow him home?</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>As Obama's Asia trip comes to a close, what's the real agenda behind his climate change focus?</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>c3_043</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Abe hopes to avoid landing in rough in golf outing with Trump</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Can a friendly game of golf help Abe smooth out a rocky relationship with Trump?</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>As Trump tees off, is the world's next president ready to sink or swim on the links with the outgoing leader?</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>c3_012</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>U.S. lawmakers deadlock on Zika virus funds</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>As Zika Virus Funding Stalls, Is Congress Running Out of Time to Protect American Families?</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>What's Holding Up the Fight Against Zika?</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>c3_002</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Facebook's Sandberg says has no plan to work in government</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>"Is Facebook's Powerhouse Leader Ruling Out a Future in Politics?".</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>What's Behind Facebook's Sheryl Sandberg's Decision to Rule Out a Government Role?</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>c3_063</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Cabinet members lobby Trump to remove Iraq from new travel ban: officials</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>"Will the White House Yield to Cabinet Pressure and Ease Restrictions on Iraq Travelers Next Week?".</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>What's behind the sudden push to exempt Iraq from the travel ban?</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>c3_061</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Michigan governor names panel to fix Flint's contaminated water system</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Whose Fix Will Flint's Poisoned Water System Get? Michigan Governor Taps a Team to Find Out.</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>What's the Plan to Finally Fix Flint's Toxic Water Crisis?</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>c3_060</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Obama, Republican leaders seek elusive common ground in White House meeting</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>What's the Secret to Bridging the Divide? Obama and GOP Leaders Meet Behind Closed Doors.</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>As Obama and Republican leaders converge on the White House, will today mark a breakthrough in their quest for common ground or another stalemate in the making?</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>c3_015</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Trump says Taiwan president 'called me' to offer congratulations</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>What prompted Taiwan's leader to reach out to the White House?</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>"Did Taiwan's leader extend a personal phone call to Trump, or was it just a routine diplomatic courtesy?".</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>c3_023</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Trump's choice for national security adviser had early exposure to Iran</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Who got a rare glimpse into Iran's inner workings before Trump's top pick took the reins?</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Whose ear did Trump's national security adviser-to-be lend to Iran's whispers early on?</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>c3_099</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>From prairie to the White House: Inside a Tribe's quest to stop a pipeline</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>What drives a tribe's determination to halt a pipeline's path from the heartland to the nation's capital?</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Whose path will be paved by progress: The pipeline's route to power or the tribe's road to resistance?</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>c3_032</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>In rural-urban divide, U.S. voters are worlds apart</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>What's driving the growing chasm between America's city dwellers and country folk?</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>As America's demographics drift apart, have rural voters and urbanites irreconcilably parted ways on election day?</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"A,B"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>